<commit_message>
motor mode and gen modes are combined
</commit_message>
<xml_diff>
--- a/PIcalc.xlsx
+++ b/PIcalc.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>fpwm</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>T</t>
+  </si>
+  <si>
+    <t>1/T</t>
   </si>
   <si>
     <t>kb</t>
@@ -1651,10 +1654,17 @@
         <f>1/B1</f>
         <v>5.0000000000000002e-05</v>
       </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <f>1/B5</f>
+        <v>20000</v>
+      </c>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <f>B3/B2</f>
@@ -1663,20 +1673,20 @@
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>20000</v>
       </c>
       <c r="D11" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E11">
         <f>B11/(2*PI())</f>
         <v>3183.098861837907</v>
       </c>
       <c r="G11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H11">
         <f>B1/E11</f>
@@ -1685,7 +1695,7 @@
     </row>
     <row r="13" ht="14.25">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B13">
         <f>B2*B11</f>
@@ -1694,7 +1704,7 @@
     </row>
     <row r="14" ht="14.25">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B14">
         <f>B10*B13</f>
@@ -1703,7 +1713,7 @@
     </row>
     <row r="17" ht="14.25">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B17">
         <f>B2/(B5)</f>
@@ -1712,7 +1722,7 @@
     </row>
     <row r="19" ht="14.25">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B19">
         <f>B17*B10</f>
@@ -1721,7 +1731,7 @@
     </row>
     <row r="21" ht="14.25">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21">
         <f>B17/B2</f>
@@ -1730,14 +1740,14 @@
     </row>
     <row r="50" ht="14.25">
       <c r="A50" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B50">
         <f>'Лист1'!B11</f>
         <v>20000</v>
       </c>
       <c r="C50" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D50">
         <f>1/B50</f>
@@ -1746,7 +1756,7 @@
     </row>
     <row r="51" ht="14.25">
       <c r="A51" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B51">
         <f>5*B50</f>
@@ -1761,7 +1771,7 @@
     </row>
     <row r="53" ht="14.25">
       <c r="A53" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B53">
         <f>B52/50</f>
@@ -1770,16 +1780,16 @@
     </row>
     <row r="54" ht="14.25">
       <c r="C54" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D54" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E54" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F54" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G54" t="s">
         <v>1</v>
@@ -1810,7 +1820,7 @@
         <v>-1.0857360059726908e-08</v>
       </c>
       <c r="J55" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="56" ht="14.25">

</xml_diff>